<commit_message>
patentes, ubicacion y parquimetro
muestra los carteles y almacena los datos pero falta comparar con la tabla si son correctos y hacer el resto
</commit_message>
<xml_diff>
--- a/Ejercicio 1/Traza.xlsx
+++ b/Ejercicio 1/Traza.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="97">
   <si>
     <t>dni</t>
   </si>
@@ -298,6 +298,15 @@
   </si>
   <si>
     <t>"12:20:01"</t>
+  </si>
+  <si>
+    <t>Estacionados</t>
+  </si>
+  <si>
+    <t>(Vista)</t>
+  </si>
+  <si>
+    <t>patente(con estacionamiento abierto en esta ubicación)</t>
   </si>
 </sst>
 </file>
@@ -481,11 +490,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -495,55 +555,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="8" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -848,7 +884,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="D7:S49"/>
+  <dimension ref="D7:S58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
@@ -858,201 +894,201 @@
   <sheetData>
     <row r="7" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="8" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="4"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="21"/>
       <c r="J8" s="1"/>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="4"/>
+      <c r="L8" s="20"/>
+      <c r="M8" s="20"/>
+      <c r="N8" s="20"/>
+      <c r="O8" s="21"/>
       <c r="P8" s="1"/>
-      <c r="Q8" s="2" t="s">
+      <c r="Q8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="R8" s="4"/>
+      <c r="R8" s="21"/>
       <c r="S8" s="1"/>
     </row>
     <row r="9" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="I9" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J9" s="1"/>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="4" t="s">
         <v>0</v>
       </c>
       <c r="P9" s="1"/>
-      <c r="Q9" s="5" t="s">
+      <c r="Q9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="R9" s="7" t="s">
+      <c r="R9" s="4" t="s">
         <v>12</v>
       </c>
       <c r="S9" s="1"/>
     </row>
     <row r="10" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D10" s="5">
+      <c r="D10" s="2">
         <v>12547879</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="3">
         <v>154879865</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="4">
         <v>450</v>
       </c>
       <c r="J10" s="1"/>
-      <c r="K10" s="5" t="s">
+      <c r="K10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="M10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="O10" s="7">
+      <c r="O10" s="4">
         <v>12547879</v>
       </c>
       <c r="P10" s="1"/>
-      <c r="Q10" s="5" t="s">
+      <c r="Q10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R10" s="7">
+      <c r="R10" s="4">
         <v>0.05</v>
       </c>
       <c r="S10" s="1"/>
     </row>
     <row r="11" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D11" s="5">
+      <c r="D11" s="2">
         <v>10458744</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="3">
         <v>159547862</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="4">
         <v>840</v>
       </c>
       <c r="J11" s="1"/>
-      <c r="K11" s="5" t="s">
+      <c r="K11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="M11" s="6" t="s">
+      <c r="M11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="N11" s="6" t="s">
+      <c r="N11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O11" s="7">
+      <c r="O11" s="4">
         <v>10458744</v>
       </c>
       <c r="P11" s="1"/>
-      <c r="Q11" s="5" t="s">
+      <c r="Q11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="R11" s="7">
+      <c r="R11" s="4">
         <v>0.3</v>
       </c>
       <c r="S11" s="1"/>
     </row>
     <row r="12" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D12" s="8">
+      <c r="D12" s="5">
         <v>40578954</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="9">
+      <c r="H12" s="6">
         <v>152124578</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="7">
         <v>320</v>
       </c>
       <c r="J12" s="1"/>
-      <c r="K12" s="8" t="s">
+      <c r="K12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="L12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="M12" s="9" t="s">
+      <c r="M12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="N12" s="9" t="s">
+      <c r="N12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="O12" s="10">
+      <c r="O12" s="7">
         <v>40578954</v>
       </c>
       <c r="P12" s="1"/>
-      <c r="Q12" s="8" t="s">
+      <c r="Q12" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="R12" s="10">
+      <c r="R12" s="7">
         <v>0.5</v>
       </c>
       <c r="S12" s="1"/>
@@ -1166,192 +1202,192 @@
       <c r="S18" s="1"/>
     </row>
     <row r="19" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="4"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="21"/>
       <c r="H19" s="1"/>
-      <c r="I19" s="2" t="s">
+      <c r="I19" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="M19" s="4"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="21"/>
       <c r="N19" s="1"/>
-      <c r="O19" s="2" t="s">
+      <c r="O19" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="4"/>
+      <c r="P19" s="20"/>
+      <c r="Q19" s="21"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
     </row>
     <row r="20" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="7" t="s">
+      <c r="G20" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H20" s="1"/>
-      <c r="I20" s="19" t="s">
+      <c r="I20" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="K20" s="20" t="s">
+      <c r="K20" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="L20" s="20" t="s">
+      <c r="L20" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="18" t="s">
         <v>43</v>
       </c>
       <c r="N20" s="1"/>
-      <c r="O20" s="19" t="s">
+      <c r="O20" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="P20" s="20" t="s">
+      <c r="P20" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="Q20" s="21" t="s">
+      <c r="Q20" s="18" t="s">
         <v>56</v>
       </c>
       <c r="R20" s="1"/>
       <c r="S20" s="1"/>
     </row>
     <row r="21" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D21" s="5">
+      <c r="D21" s="2">
         <v>1212</v>
       </c>
-      <c r="E21" s="6">
+      <c r="E21" s="3">
         <v>450.01</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="4" t="s">
         <v>18</v>
       </c>
       <c r="H21" s="1"/>
-      <c r="I21" s="5">
+      <c r="I21" s="2">
         <v>12</v>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="3">
         <v>15487612</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="K21" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="M21" s="7" t="s">
+      <c r="M21" s="4" t="s">
         <v>51</v>
       </c>
       <c r="N21" s="1"/>
-      <c r="O21" s="5" t="s">
+      <c r="O21" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="P21" s="6">
+      <c r="P21" s="3">
         <v>1000</v>
       </c>
-      <c r="Q21" s="7">
+      <c r="Q21" s="4">
         <v>100.05</v>
       </c>
       <c r="R21" s="1"/>
       <c r="S21" s="1"/>
     </row>
     <row r="22" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D22" s="5">
+      <c r="D22" s="2">
         <v>5487</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="3">
         <v>870.95</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H22" s="1"/>
-      <c r="I22" s="5">
+      <c r="I22" s="2">
         <v>13</v>
       </c>
-      <c r="J22" s="6">
+      <c r="J22" s="3">
         <v>40874125</v>
       </c>
-      <c r="K22" s="6" t="s">
+      <c r="K22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="L22" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="M22" s="7" t="s">
+      <c r="M22" s="4" t="s">
         <v>52</v>
       </c>
       <c r="N22" s="1"/>
-      <c r="O22" s="5" t="s">
+      <c r="O22" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="P22" s="6">
+      <c r="P22" s="3">
         <v>200</v>
       </c>
-      <c r="Q22" s="7">
+      <c r="Q22" s="4">
         <v>150.05000000000001</v>
       </c>
       <c r="R22" s="1"/>
       <c r="S22" s="1"/>
     </row>
     <row r="23" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D23" s="8">
+      <c r="D23" s="5">
         <v>6598</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="6">
         <v>140.15</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="F23" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" s="7" t="s">
         <v>20</v>
       </c>
       <c r="H23" s="1"/>
-      <c r="I23" s="8">
+      <c r="I23" s="5">
         <v>14</v>
       </c>
-      <c r="J23" s="9">
+      <c r="J23" s="6">
         <v>25604782</v>
       </c>
-      <c r="K23" s="9" t="s">
+      <c r="K23" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="L23" s="9" t="s">
+      <c r="L23" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="M23" s="10" t="s">
+      <c r="M23" s="7" t="s">
         <v>53</v>
       </c>
       <c r="N23" s="1"/>
-      <c r="O23" s="8" t="s">
+      <c r="O23" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="P23" s="9">
+      <c r="P23" s="6">
         <v>100</v>
       </c>
-      <c r="Q23" s="10">
+      <c r="Q23" s="7">
         <v>248.04</v>
       </c>
       <c r="R23" s="1"/>
@@ -1484,210 +1520,210 @@
       <c r="S30" s="1"/>
     </row>
     <row r="31" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="4"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
+      <c r="G31" s="21"/>
       <c r="H31" s="1"/>
-      <c r="I31" s="2" t="s">
+      <c r="I31" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="J31" s="3"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="3"/>
-      <c r="M31" s="3"/>
-      <c r="N31" s="4"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="20"/>
+      <c r="L31" s="20"/>
+      <c r="M31" s="20"/>
+      <c r="N31" s="21"/>
       <c r="O31" s="1"/>
-      <c r="P31" s="2" t="s">
+      <c r="P31" s="19" t="s">
         <v>76</v>
       </c>
-      <c r="Q31" s="3"/>
-      <c r="R31" s="3"/>
-      <c r="S31" s="4"/>
+      <c r="Q31" s="20"/>
+      <c r="R31" s="20"/>
+      <c r="S31" s="21"/>
     </row>
     <row r="32" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G32" s="4" t="s">
         <v>55</v>
       </c>
       <c r="H32" s="1"/>
-      <c r="I32" s="5" t="s">
+      <c r="I32" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="M32" s="6" t="s">
+      <c r="M32" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="N32" s="7" t="s">
+      <c r="N32" s="4" t="s">
         <v>67</v>
       </c>
       <c r="O32" s="1"/>
-      <c r="P32" s="5" t="s">
+      <c r="P32" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Q32" s="6" t="s">
+      <c r="Q32" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="R32" s="6" t="s">
+      <c r="R32" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="S32" s="7" t="s">
+      <c r="S32" s="4" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="33" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D33" s="5">
+      <c r="D33" s="2">
         <v>150</v>
       </c>
-      <c r="E33" s="6">
+      <c r="E33" s="3">
         <v>1</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="7">
+      <c r="G33" s="4">
         <v>1000</v>
       </c>
       <c r="H33" s="1"/>
-      <c r="I33" s="5">
+      <c r="I33" s="2">
         <v>1212</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="3">
         <v>150</v>
       </c>
-      <c r="K33" s="15" t="s">
+      <c r="K33" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="L33" s="12" t="s">
+      <c r="L33" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="M33" s="12" t="s">
+      <c r="M33" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="N33" s="16" t="s">
+      <c r="N33" s="13" t="s">
         <v>89</v>
       </c>
       <c r="O33" s="1"/>
-      <c r="P33" s="5">
+      <c r="P33" s="2">
         <v>12</v>
       </c>
-      <c r="Q33" s="6">
+      <c r="Q33" s="3">
         <v>150</v>
       </c>
-      <c r="R33" s="15" t="s">
+      <c r="R33" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="S33" s="16" t="s">
+      <c r="S33" s="13" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="34" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D34" s="5">
+      <c r="D34" s="2">
         <v>120</v>
       </c>
-      <c r="E34" s="6">
+      <c r="E34" s="3">
         <v>2</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="F34" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="4">
         <v>200</v>
       </c>
       <c r="H34" s="1"/>
-      <c r="I34" s="5">
+      <c r="I34" s="2">
         <v>5487</v>
       </c>
-      <c r="J34" s="6">
+      <c r="J34" s="3">
         <v>120</v>
       </c>
-      <c r="K34" s="15" t="s">
+      <c r="K34" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="L34" s="12" t="s">
+      <c r="L34" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="M34" s="12" t="s">
+      <c r="M34" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="N34" s="16" t="s">
+      <c r="N34" s="13" t="s">
         <v>90</v>
       </c>
       <c r="O34" s="1"/>
-      <c r="P34" s="5">
+      <c r="P34" s="2">
         <v>13</v>
       </c>
-      <c r="Q34" s="6">
+      <c r="Q34" s="3">
         <v>120</v>
       </c>
-      <c r="R34" s="15" t="s">
+      <c r="R34" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="S34" s="16" t="s">
+      <c r="S34" s="13" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="35" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D35" s="8">
+      <c r="D35" s="5">
         <v>190</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E35" s="6">
         <v>3</v>
       </c>
-      <c r="F35" s="9" t="s">
+      <c r="F35" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G35" s="10">
+      <c r="G35" s="7">
         <v>100</v>
       </c>
       <c r="H35" s="1"/>
-      <c r="I35" s="8">
+      <c r="I35" s="5">
         <v>6598</v>
       </c>
-      <c r="J35" s="9">
+      <c r="J35" s="6">
         <v>190</v>
       </c>
-      <c r="K35" s="17" t="s">
+      <c r="K35" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="L35" s="13" t="s">
+      <c r="L35" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="M35" s="13" t="s">
+      <c r="M35" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="N35" s="18" t="s">
+      <c r="N35" s="15" t="s">
         <v>90</v>
       </c>
       <c r="O35" s="1"/>
-      <c r="P35" s="8">
+      <c r="P35" s="5">
         <v>14</v>
       </c>
-      <c r="Q35" s="9">
+      <c r="Q35" s="6">
         <v>190</v>
       </c>
-      <c r="R35" s="17" t="s">
+      <c r="R35" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="S35" s="18" t="s">
+      <c r="S35" s="15" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1800,182 +1836,182 @@
       <c r="S41" s="1"/>
     </row>
     <row r="42" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D42" s="2" t="s">
+      <c r="D42" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="E42" s="3"/>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="4"/>
+      <c r="E42" s="20"/>
+      <c r="F42" s="20"/>
+      <c r="G42" s="20"/>
+      <c r="H42" s="20"/>
+      <c r="I42" s="21"/>
       <c r="J42" s="1"/>
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
-      <c r="M42" s="2" t="s">
+      <c r="M42" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="N42" s="3"/>
-      <c r="O42" s="3"/>
-      <c r="P42" s="3"/>
-      <c r="Q42" s="4"/>
-      <c r="R42" s="11"/>
+      <c r="N42" s="20"/>
+      <c r="O42" s="20"/>
+      <c r="P42" s="20"/>
+      <c r="Q42" s="21"/>
+      <c r="R42" s="8"/>
       <c r="S42" s="1"/>
     </row>
     <row r="43" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D43" s="5" t="s">
+      <c r="D43" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E43" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="F43" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="G43" s="6" t="s">
+      <c r="G43" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H43" s="6" t="s">
+      <c r="H43" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I43" s="7" t="s">
+      <c r="I43" s="4" t="s">
         <v>73</v>
       </c>
       <c r="J43" s="1"/>
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
-      <c r="M43" s="5" t="s">
+      <c r="M43" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="N43" s="6" t="s">
+      <c r="N43" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="O43" s="6" t="s">
+      <c r="O43" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="P43" s="6" t="s">
+      <c r="P43" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="Q43" s="7" t="s">
+      <c r="Q43" s="4" t="s">
         <v>71</v>
       </c>
       <c r="R43" s="1"/>
       <c r="S43" s="1"/>
     </row>
     <row r="44" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D44" s="5">
+      <c r="D44" s="2">
         <v>5050</v>
       </c>
-      <c r="E44" s="6">
+      <c r="E44" s="3">
         <v>12</v>
       </c>
-      <c r="F44" s="6" t="s">
+      <c r="F44" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="G44" s="6">
+      <c r="G44" s="3">
         <v>1000</v>
       </c>
-      <c r="H44" s="14" t="s">
+      <c r="H44" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="I44" s="7" t="s">
+      <c r="I44" s="4" t="s">
         <v>80</v>
       </c>
       <c r="J44" s="1"/>
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
-      <c r="M44" s="5">
+      <c r="M44" s="2">
         <v>115</v>
       </c>
-      <c r="N44" s="15" t="s">
+      <c r="N44" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="O44" s="12" t="s">
+      <c r="O44" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="P44" s="6" t="s">
+      <c r="P44" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="Q44" s="7">
+      <c r="Q44" s="4">
         <v>5050</v>
       </c>
       <c r="R44" s="1"/>
       <c r="S44" s="1"/>
     </row>
     <row r="45" spans="4:19" x14ac:dyDescent="0.25">
-      <c r="D45" s="5">
+      <c r="D45" s="2">
         <v>6060</v>
       </c>
-      <c r="E45" s="6">
+      <c r="E45" s="3">
         <v>13</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="F45" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="G45" s="6">
+      <c r="G45" s="3">
         <v>200</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="H45" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="I45" s="7" t="s">
+      <c r="I45" s="4" t="s">
         <v>81</v>
       </c>
       <c r="J45" s="1"/>
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
-      <c r="M45" s="5">
+      <c r="M45" s="2">
         <v>116</v>
       </c>
-      <c r="N45" s="15" t="s">
+      <c r="N45" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="O45" s="12" t="s">
+      <c r="O45" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="P45" s="6" t="s">
+      <c r="P45" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="Q45" s="7">
+      <c r="Q45" s="4">
         <v>6060</v>
       </c>
       <c r="R45" s="1"/>
       <c r="S45" s="1"/>
     </row>
     <row r="46" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D46" s="8">
+      <c r="D46" s="5">
         <v>7070</v>
       </c>
-      <c r="E46" s="9">
+      <c r="E46" s="6">
         <v>14</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="F46" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="G46" s="9">
+      <c r="G46" s="6">
         <v>100</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H46" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="I46" s="10" t="s">
+      <c r="I46" s="7" t="s">
         <v>80</v>
       </c>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
-      <c r="M46" s="8">
+      <c r="M46" s="5">
         <v>117</v>
       </c>
-      <c r="N46" s="17" t="s">
+      <c r="N46" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="O46" s="13" t="s">
+      <c r="O46" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="P46" s="9" t="s">
+      <c r="P46" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="Q46" s="10">
+      <c r="Q46" s="7">
         <v>7070</v>
       </c>
       <c r="R46" s="1"/>
@@ -2035,19 +2071,100 @@
       <c r="R49" s="1"/>
       <c r="S49" s="1"/>
     </row>
+    <row r="53" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H53" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="54" spans="4:19" x14ac:dyDescent="0.25">
+      <c r="G54" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="H54" s="23"/>
+      <c r="I54" s="23"/>
+      <c r="J54" s="23"/>
+      <c r="K54" s="23"/>
+      <c r="L54" s="23"/>
+      <c r="M54" s="24"/>
+    </row>
+    <row r="55" spans="4:19" x14ac:dyDescent="0.25">
+      <c r="G55" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I55" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="J55" s="29"/>
+      <c r="K55" s="29"/>
+      <c r="L55" s="29"/>
+      <c r="M55" s="30"/>
+    </row>
+    <row r="56" spans="4:19" x14ac:dyDescent="0.25">
+      <c r="G56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H56" s="3">
+        <v>1000</v>
+      </c>
+      <c r="I56" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="J56" s="25"/>
+      <c r="K56" s="25"/>
+      <c r="L56" s="25"/>
+      <c r="M56" s="26"/>
+    </row>
+    <row r="57" spans="4:19" x14ac:dyDescent="0.25">
+      <c r="G57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H57" s="3">
+        <v>200</v>
+      </c>
+      <c r="I57" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="J57" s="25"/>
+      <c r="K57" s="25"/>
+      <c r="L57" s="25"/>
+      <c r="M57" s="26"/>
+    </row>
+    <row r="58" spans="4:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G58" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H58" s="6">
+        <v>100</v>
+      </c>
+      <c r="I58" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J58" s="27"/>
+      <c r="K58" s="27"/>
+      <c r="L58" s="27"/>
+      <c r="M58" s="28"/>
+    </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="I31:N31"/>
-    <mergeCell ref="D42:I42"/>
-    <mergeCell ref="P31:S31"/>
-    <mergeCell ref="M42:Q42"/>
+  <mergeCells count="16">
+    <mergeCell ref="G54:M54"/>
+    <mergeCell ref="I55:M55"/>
+    <mergeCell ref="I58:M58"/>
+    <mergeCell ref="I57:M57"/>
+    <mergeCell ref="I56:M56"/>
     <mergeCell ref="D8:I8"/>
     <mergeCell ref="K8:O8"/>
     <mergeCell ref="Q8:R8"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="I19:M19"/>
     <mergeCell ref="O19:Q19"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="I31:N31"/>
+    <mergeCell ref="D42:I42"/>
+    <mergeCell ref="P31:S31"/>
+    <mergeCell ref="M42:Q42"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>